<commit_message>
Add prediction graph template and integrate into various pages
- Introduced a new template for displaying prediction graphs.
- Updated base styles for improved UI consistency.
- Integrated prediction graph into the dashboard, chits, entity list, overall assets, paired workspace, and sneha payments pages.
- Enhanced the dashboard hero section with updated descriptions and actions.
- Refined the layout and styles for better responsiveness and visual appeal.
- Adjusted logic for displaying mutual fund counts and scheme configurations in the paired workspace.
</commit_message>
<xml_diff>
--- a/financial_dashboard/Income.xlsx
+++ b/financial_dashboard/Income.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venka\Desktop\Income\income\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77B1716A-BF38-443B-9EE7-8C3BEA01239C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B632586-D5BF-42FB-BC1E-6198437682F4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Banks" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="274">
   <si>
     <t>id</t>
   </si>
@@ -864,6 +864,9 @@
   </si>
   <si>
     <t>days diffrence</t>
+  </si>
+  <si>
+    <t>Column1</t>
   </si>
 </sst>
 </file>
@@ -993,7 +996,19 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="40">
+  <dxfs count="41">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1060,22 +1075,13 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1176,7 +1182,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B31CE97E-6A8E-498A-9DE7-CAB216D91CDE}" name="Table1" displayName="Table1" ref="A1:B6" totalsRowShown="0">
   <autoFilter ref="A1:B6" xr:uid="{8CFA6E78-CFEB-47EF-86DF-451D9C230FDC}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DB3A3612-B83E-4D7B-B254-D5E87FA9835F}" name="id" dataDxfId="39"/>
+    <tableColumn id="1" xr3:uid="{DB3A3612-B83E-4D7B-B254-D5E87FA9835F}" name="id" dataDxfId="40"/>
     <tableColumn id="2" xr3:uid="{85D7CF35-0544-42D5-972C-21C95C59C0E4}" name="name"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1188,7 +1194,7 @@
   <autoFilter ref="A1:D7" xr:uid="{00A1A986-D773-4AC7-9248-5655021C7C04}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{60E2BE4A-BF9C-4F63-AF90-CAE2E411C201}" name="Spending Type"/>
-    <tableColumn id="2" xr3:uid="{4E026AD4-5C62-4EE5-B4AD-39440802E3F9}" name="Amount" totalsRowFunction="custom" dataDxfId="3" totalsRowDxfId="2">
+    <tableColumn id="2" xr3:uid="{4E026AD4-5C62-4EE5-B4AD-39440802E3F9}" name="Amount" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
       <totalsRowFormula>SUM(Table6[Amount])</totalsRowFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{63CA58E3-4990-483C-8F2E-7A687EBE2722}" name="Person"/>
@@ -1203,7 +1209,7 @@
   <autoFilter ref="A1:B7" xr:uid="{E75938B2-6DD9-4A29-BA86-8D8B50A6C9F4}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{DF10BC0A-2099-4906-A7AB-62C0916746B3}" name="Label"/>
-    <tableColumn id="2" xr3:uid="{848C545C-47EE-4883-AE2A-B47C8FCE9A59}" name="Amount" totalsRowFunction="custom" dataDxfId="1" totalsRowDxfId="0">
+    <tableColumn id="2" xr3:uid="{848C545C-47EE-4883-AE2A-B47C8FCE9A59}" name="Amount" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
       <totalsRowFormula>SUM(Table12[Amount])</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -1215,7 +1221,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B44E878A-10A6-457B-B8C3-51324B90DAB2}" name="Table2" displayName="Table2" ref="A1:O3" totalsRowShown="0">
   <autoFilter ref="A1:O3" xr:uid="{8C15CAC8-E359-4B6E-8B28-9630C48729AF}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{FBA81958-7492-4F54-8F4A-25EFCF6A5B4D}" name="id" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{FBA81958-7492-4F54-8F4A-25EFCF6A5B4D}" name="id" dataDxfId="39"/>
     <tableColumn id="2" xr3:uid="{5FD37CCE-BA6A-43C8-9E9B-83A7A4EA08C8}" name="full_name"/>
     <tableColumn id="3" xr3:uid="{4A844664-C67F-428B-BB85-EF5C01D52A7E}" name="username"/>
     <tableColumn id="4" xr3:uid="{86EABDC0-DD78-477C-938E-6F40F48EFEDA}" name="email"/>
@@ -1239,10 +1245,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3981DD6A-2D42-43D9-95EE-9724BCCA7483}" name="Table3" displayName="Table3" ref="A1:E8" totalsRowCount="1">
   <autoFilter ref="A1:E7" xr:uid="{8F00FFC1-A830-480F-BD36-4C288E783DEE}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{FC72FF4D-248D-4291-B7A0-6A90DFF0EA3F}" name="id" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{BFA836AD-0FD0-470C-9574-040D8E8CF44A}" name="user_id" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{1BC58DB4-B1A5-4793-9894-20379173207B}" name="bank_id" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{90F6EA90-A9BC-4549-9C1A-6B8CE3C5CAF1}" name="balance" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
+    <tableColumn id="1" xr3:uid="{FC72FF4D-248D-4291-B7A0-6A90DFF0EA3F}" name="id" dataDxfId="38" totalsRowDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{BFA836AD-0FD0-470C-9574-040D8E8CF44A}" name="user_id" dataDxfId="37" totalsRowDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{1BC58DB4-B1A5-4793-9894-20379173207B}" name="bank_id" dataDxfId="36" totalsRowDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{90F6EA90-A9BC-4549-9C1A-6B8CE3C5CAF1}" name="balance" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="0">
       <totalsRowFormula>SUM(Table3[balance])</totalsRowFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{AF74AA07-F182-42F3-8828-C32E6786C2E3}" name="purpose"/>
@@ -1255,25 +1261,25 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3B211DA3-508F-49BD-BDC8-8A70246CE88B}" name="Table4" displayName="Table4" ref="A1:K36" totalsRowShown="0">
   <autoFilter ref="A1:K36" xr:uid="{8DFC41D8-64F7-4568-9581-A4A165E6C8FF}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{5E359C7C-6644-422F-B05C-8EF48D69F367}" name="S.No" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{757C3E82-48B9-41DB-B1FA-CD13752BF34E}" name="account_id" dataDxfId="27" totalsRowDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{42B47B3A-95C3-4DE8-8220-39183DBF3468}" name="Invested" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{C7366A70-35D3-4800-8A09-515BC5388DBD}" name="Interest Rate" dataDxfId="24" totalsRowDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{5E359C7C-6644-422F-B05C-8EF48D69F367}" name="S.No" dataDxfId="34" totalsRowDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{757C3E82-48B9-41DB-B1FA-CD13752BF34E}" name="account_id" dataDxfId="32" totalsRowDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{42B47B3A-95C3-4DE8-8220-39183DBF3468}" name="Invested" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{C7366A70-35D3-4800-8A09-515BC5388DBD}" name="Interest Rate" dataDxfId="29" totalsRowDxfId="28"/>
     <tableColumn id="5" xr3:uid="{5D3560D2-531B-4762-9769-E8ACD64F4761}" name="Maturity Date"/>
     <tableColumn id="6" xr3:uid="{997B0C2C-3B66-43E1-B495-C5D1BA4E2C11}" name="Created Date"/>
-    <tableColumn id="7" xr3:uid="{8999C824-07CA-48FC-9C7E-DAE9CDF5B7FD}" name="TODAY" dataDxfId="22" totalsRowDxfId="21">
+    <tableColumn id="7" xr3:uid="{8999C824-07CA-48FC-9C7E-DAE9CDF5B7FD}" name="TODAY" dataDxfId="27" totalsRowDxfId="26">
       <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{9BF25733-5C68-4283-A5CC-76E58A86F7AF}" name="Current Amount" dataDxfId="20">
+    <tableColumn id="8" xr3:uid="{9BF25733-5C68-4283-A5CC-76E58A86F7AF}" name="Current Amount" dataDxfId="25">
       <calculatedColumnFormula>(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{954CBA2A-5592-4248-A149-91CB2BDB7B35}" name="Days To Mature" dataDxfId="19" totalsRowDxfId="18">
+    <tableColumn id="9" xr3:uid="{954CBA2A-5592-4248-A149-91CB2BDB7B35}" name="Days To Mature" dataDxfId="24" totalsRowDxfId="23">
       <calculatedColumnFormula>E2-G2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BC9C4C9A-966B-47E0-A258-D56038E8A995}" name="invested days" dataDxfId="17">
+    <tableColumn id="10" xr3:uid="{BC9C4C9A-966B-47E0-A258-D56038E8A995}" name="invested days" dataDxfId="22">
       <calculatedColumnFormula>_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{C306C9AC-2771-4EAE-99E2-80D6769E204B}" name="days diffrence" dataDxfId="16">
+    <tableColumn id="11" xr3:uid="{C306C9AC-2771-4EAE-99E2-80D6769E204B}" name="days diffrence" dataDxfId="21">
       <calculatedColumnFormula>I2-I1</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1282,9 +1288,12 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1424231E-1A3B-4998-877B-E5561215BA59}" name="Table5" displayName="Table5" ref="A1:J22" totalsRowShown="0">
-  <autoFilter ref="A1:J22" xr:uid="{1A2C2465-CFFA-4132-B427-2BF57C3D84EE}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1424231E-1A3B-4998-877B-E5561215BA59}" name="Table5" displayName="Table5" ref="A1:K22" totalsRowShown="0">
+  <autoFilter ref="A1:K22" xr:uid="{1A2C2465-CFFA-4132-B427-2BF57C3D84EE}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K22">
+    <sortCondition descending="1" ref="K1:K22"/>
+  </sortState>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{29392632-74D8-4C1F-982A-2E95DF6BEE86}" name="S.No"/>
     <tableColumn id="2" xr3:uid="{CDDAF558-A430-476F-9C24-1857E98B1E8B}" name="Symbol"/>
     <tableColumn id="3" xr3:uid="{42D1F168-99E0-418A-9E3E-0115448812A7}" name="Exchange"/>
@@ -1293,11 +1302,14 @@
     <tableColumn id="6" xr3:uid="{3526CB46-6BC5-409C-A88C-2D55CD654C35}" name="Current Price"/>
     <tableColumn id="7" xr3:uid="{1082033A-DCD1-4110-8874-1DC66CCF7D7B}" name="Quantity"/>
     <tableColumn id="8" xr3:uid="{CC1FA5FC-72F1-427E-8427-FF420DE8A3CD}" name="Source"/>
-    <tableColumn id="9" xr3:uid="{5A1BC9AB-281D-447D-94A7-1ECD62B6C06C}" name="Invested" dataDxfId="15">
+    <tableColumn id="9" xr3:uid="{5A1BC9AB-281D-447D-94A7-1ECD62B6C06C}" name="Invested" dataDxfId="20">
       <calculatedColumnFormula>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{E93CFF81-628F-46A7-B0AA-3EAAFA5C292F}" name="current" dataDxfId="14">
+    <tableColumn id="10" xr3:uid="{E93CFF81-628F-46A7-B0AA-3EAAFA5C292F}" name="current" dataDxfId="19">
       <calculatedColumnFormula>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{4DC395D2-53E8-42CC-AFBD-675876AA0876}" name="Column1" dataDxfId="18">
+      <calculatedColumnFormula>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1305,10 +1317,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B55F72A0-DB12-4984-862F-5C53E962E94A}" name="Table7" displayName="Table7" ref="A1:L11" totalsRowShown="0" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B55F72A0-DB12-4984-862F-5C53E962E94A}" name="Table7" displayName="Table7" ref="A1:L11" totalsRowShown="0" dataDxfId="17">
   <autoFilter ref="A1:L11" xr:uid="{6F644203-C1C1-4DB2-9663-46291F68AFE7}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{F127C49A-C2F6-46E9-8F53-BAFE036ED111}" name="S.No" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{F127C49A-C2F6-46E9-8F53-BAFE036ED111}" name="S.No" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{4642C1C5-D86D-4BD6-A9A3-9DA679706C1A}" name="id"/>
     <tableColumn id="3" xr3:uid="{EA5A4C19-74EA-4D52-87D8-D0A3F5D33B55}" name="fund_name"/>
     <tableColumn id="4" xr3:uid="{5A2E588B-26BE-4722-A596-0E368C770D52}" name="scheme_code"/>
@@ -1318,10 +1330,10 @@
     <tableColumn id="8" xr3:uid="{C638FFDA-94ED-4D91-B8C3-149B9085BF53}" name="latest_nav"/>
     <tableColumn id="9" xr3:uid="{0151F1C5-532C-4D98-94D9-CE34BC112438}" name="nav_date"/>
     <tableColumn id="10" xr3:uid="{69731B32-5278-4E4E-B3A2-6F1A95D14679}" name="sip"/>
-    <tableColumn id="11" xr3:uid="{95D0BA28-5DF9-4BE2-8BF7-C2C1ED0C5084}" name="Invested" dataDxfId="11">
+    <tableColumn id="11" xr3:uid="{95D0BA28-5DF9-4BE2-8BF7-C2C1ED0C5084}" name="Invested" dataDxfId="15">
       <calculatedColumnFormula>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{A098199E-E9C3-4E6A-AF5B-15CD0322630E}" name="Current" dataDxfId="10">
+    <tableColumn id="12" xr3:uid="{A098199E-E9C3-4E6A-AF5B-15CD0322630E}" name="Current" dataDxfId="14">
       <calculatedColumnFormula>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1345,12 +1357,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{E1B721C6-8217-46EA-9CB6-12659F2BFC36}" name="Table9" displayName="Table9" ref="A1:D9" totalsRowCount="1">
   <autoFilter ref="A1:D8" xr:uid="{111C8EBC-7A2D-4CC5-A879-75B1BAA7645D}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{EB4348AE-6EC0-47B2-8224-999A95CE310F}" name="S.No" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{EB4348AE-6EC0-47B2-8224-999A95CE310F}" name="S.No" dataDxfId="13" totalsRowDxfId="6"/>
     <tableColumn id="2" xr3:uid="{AC15ADE5-1353-4EEA-BE04-4B277C82DC60}" name="Borrower"/>
-    <tableColumn id="3" xr3:uid="{1DDDBFCD-4BB8-4C8E-B682-60CC0968DEA9}" name="Amount" totalsRowFunction="custom" dataDxfId="7" totalsRowDxfId="6">
+    <tableColumn id="3" xr3:uid="{1DDDBFCD-4BB8-4C8E-B682-60CC0968DEA9}" name="Amount" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="5">
       <totalsRowFormula>SUM(Table9[Amount])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{3DBBC7D7-BA0C-4564-98C3-ECA9A6F6FA5F}" name="Interest Rate" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{3DBBC7D7-BA0C-4564-98C3-ECA9A6F6FA5F}" name="Interest Rate" dataDxfId="11" totalsRowDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2045,17 +2057,17 @@
       </c>
       <c r="E2" s="8">
         <f>SUM(B6:B30)</f>
-        <v>161240</v>
+        <v>187440</v>
       </c>
       <c r="F2" s="9">
         <v>45207</v>
       </c>
       <c r="G2" s="8">
         <f>B2/C2*H2</f>
-        <v>181920</v>
+        <v>212240</v>
       </c>
       <c r="H2" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2174,6 +2186,12 @@
     <row r="12" spans="1:8">
       <c r="A12" s="8">
         <v>7</v>
+      </c>
+      <c r="B12" s="8">
+        <v>26200</v>
+      </c>
+      <c r="C12" s="9">
+        <v>46150</v>
       </c>
       <c r="F12" s="8">
         <v>25440</v>
@@ -2751,7 +2769,7 @@
       </c>
       <c r="B2" s="1">
         <f ca="1">'Fixed Deposit'!H39</f>
-        <v>4707387.3958356157</v>
+        <v>4713240.9151232885</v>
       </c>
       <c r="C2" t="s">
         <v>27</v>
@@ -2766,7 +2784,7 @@
       </c>
       <c r="B3" s="1">
         <f>Table3[[#Totals],[balance]]</f>
-        <v>335227.95999999996</v>
+        <v>160592.95999999999</v>
       </c>
       <c r="C3" t="s">
         <v>27</v>
@@ -2781,7 +2799,7 @@
       </c>
       <c r="B4" s="1">
         <f>'Mutal Funds'!L13</f>
-        <v>961172.5728637001</v>
+        <v>1006237.7117467999</v>
       </c>
       <c r="C4" t="s">
         <v>27</v>
@@ -2796,7 +2814,7 @@
       </c>
       <c r="B5" s="1">
         <f>Stocks!J25</f>
-        <v>734243.99180970306</v>
+        <v>752858.34342878871</v>
       </c>
       <c r="C5" t="s">
         <v>27</v>
@@ -2811,7 +2829,7 @@
       </c>
       <c r="B6" s="1">
         <f>Loans!C9</f>
-        <v>3336602.75</v>
+        <v>3364343.45</v>
       </c>
       <c r="C6" t="s">
         <v>27</v>
@@ -2826,7 +2844,7 @@
       </c>
       <c r="B7" s="1">
         <f ca="1">Standard_Chits!I4+Variable_Chit!G2</f>
-        <v>936420</v>
+        <v>966740</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -2838,13 +2856,13 @@
     <row r="8" spans="1:8">
       <c r="B8" s="1">
         <f ca="1">SUM(Table12[Amount])</f>
-        <v>11011054.670509018</v>
+        <v>10964013.380298877</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="H10">
         <f ca="1">B2+B3+B7+SUM(Loans!C2:C6)+2100000+8000000</f>
-        <v>18252732.105835617</v>
+        <v>18142011.325123288</v>
       </c>
     </row>
   </sheetData>
@@ -2974,11 +2992,11 @@
       </c>
       <c r="B12" s="3">
         <f>C12*0.08</f>
-        <v>76893.805829096003</v>
+        <v>80499.016939743989</v>
       </c>
       <c r="C12" s="3">
         <f>'Mutal Funds'!L13</f>
-        <v>961172.5728637001</v>
+        <v>1006237.7117467999</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2987,11 +3005,11 @@
       </c>
       <c r="B13" s="3">
         <f>C13*0.1</f>
-        <v>73424.399180970315</v>
+        <v>75285.834342878879</v>
       </c>
       <c r="C13" s="3">
         <f>Stocks!J25</f>
-        <v>734243.99180970306</v>
+        <v>752858.34342878871</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -3022,17 +3040,17 @@
     <row r="16" spans="1:5">
       <c r="E16" s="3">
         <f>SUM(B10:B15)</f>
-        <v>1228239.0690100663</v>
+        <v>1233705.7152826227</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="E17" s="14">
         <f>SUM(E8,E16)</f>
-        <v>5038157.2840100657</v>
+        <v>5043623.9302826226</v>
       </c>
       <c r="G17" s="3">
         <f>E17*0.7/12</f>
-        <v>293892.5082339205</v>
+        <v>294211.39593315293</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -3105,7 +3123,7 @@
     <row r="31" spans="1:7">
       <c r="B31" s="14">
         <f>SUM(B1:B24)</f>
-        <v>6938349.2840100657</v>
+        <v>6943815.9302826235</v>
       </c>
     </row>
   </sheetData>
@@ -3321,7 +3339,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="1">
-        <v>214084.61</v>
+        <v>66449.61</v>
       </c>
       <c r="E2" t="s">
         <v>40</v>
@@ -3338,7 +3356,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="1">
-        <v>30086.6</v>
+        <v>3086.6</v>
       </c>
       <c r="E3" t="s">
         <v>38</v>
@@ -3418,7 +3436,7 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1">
         <f>SUM(Table3[balance])</f>
-        <v>335227.95999999996</v>
+        <v>160592.95999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3500,22 +3518,22 @@
       </c>
       <c r="G2" s="4">
         <f ca="1">TODAY()</f>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H2" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>111032.76712328767</v>
+        <v>111186</v>
       </c>
       <c r="I2" s="1">
         <f ca="1">E2-G2</f>
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="J2">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="K2" s="1">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -3539,19 +3557,19 @@
       </c>
       <c r="G3" s="4">
         <f t="shared" ref="G3:G36" ca="1" si="0">TODAY()</f>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H3" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>111010.87671232877</v>
+        <v>111164.10958904109</v>
       </c>
       <c r="I3" s="1">
         <f t="shared" ref="I3:I36" ca="1" si="1">E3-G3</f>
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="J3">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="K3" s="1">
         <f t="shared" ref="K3:K36" ca="1" si="2">I3-I2</f>
@@ -3579,19 +3597,19 @@
       </c>
       <c r="G4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H4" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>83797.176657534248</v>
+        <v>83913.476767123284</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="J4">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="K4" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3619,19 +3637,19 @@
       </c>
       <c r="G5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H5" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>109931.50684931508</v>
+        <v>110070.54794520549</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J5">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="K5" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3659,19 +3677,19 @@
       </c>
       <c r="G6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H6" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>106079.45205479451</v>
+        <v>106213.69863013699</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="J6">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="K6" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3699,19 +3717,19 @@
       </c>
       <c r="G7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H7" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>105810.95890410959</v>
+        <v>105945.20547945205</v>
       </c>
       <c r="I7" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="J7">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="K7" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3739,19 +3757,19 @@
       </c>
       <c r="G8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H8" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>106079.45205479451</v>
+        <v>106213.69863013699</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="J8">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="K8" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3779,19 +3797,19 @@
       </c>
       <c r="G9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H9" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>106079.45205479451</v>
+        <v>106213.69863013699</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="J9">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="K9" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3819,19 +3837,19 @@
       </c>
       <c r="G10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H10" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>106305.75342465754</v>
+        <v>106437.12328767123</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="J10">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="K10" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3859,19 +3877,19 @@
       </c>
       <c r="G11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H11" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>112082.19178082192</v>
+        <v>112216.43835616438</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="J11">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>630</v>
+        <v>637</v>
       </c>
       <c r="K11" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3899,19 +3917,19 @@
       </c>
       <c r="G12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H12" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>104967.12328767123</v>
+        <v>105101.36986301369</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="J12">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="K12" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3939,19 +3957,19 @@
       </c>
       <c r="G13" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H13" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>106305.75342465754</v>
+        <v>106437.12328767123</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="J13">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="K13" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -3979,19 +3997,19 @@
       </c>
       <c r="G14" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H14" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>101890.4109589041</v>
+        <v>102000.68493150685</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="J14">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="K14" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4019,19 +4037,19 @@
       </c>
       <c r="G15" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H15" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>101890.4109589041</v>
+        <v>102000.68493150685</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="J15">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="K15" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4059,19 +4077,19 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H16" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>102219.17808219178</v>
+        <v>102348.63013698631</v>
       </c>
       <c r="I16" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="J16">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="K16" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4099,19 +4117,19 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H17" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>203587.67123287672</v>
+        <v>203846.57534246575</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="J17">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="K17" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4139,19 +4157,19 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H18" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>102219.17808219178</v>
+        <v>102348.63013698631</v>
       </c>
       <c r="I18" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="J18">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="K18" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4179,19 +4197,19 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H19" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>204109.5890410959</v>
+        <v>204349.31506849316</v>
       </c>
       <c r="I19" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="J19">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="K19" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4219,19 +4237,19 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H20" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>102054.79452054795</v>
+        <v>102174.65753424658</v>
       </c>
       <c r="I20" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="J20">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="K20" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4259,19 +4277,19 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H21" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>152285.95890410958</v>
+        <v>152465.75342465754</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="J21">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="K21" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4299,19 +4317,19 @@
       </c>
       <c r="G22" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H22" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>102087.67123287672</v>
+        <v>102209.45205479451</v>
       </c>
       <c r="I22" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="J22">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="K22" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4339,19 +4357,19 @@
       </c>
       <c r="G23" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H23" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>152311.64383561644</v>
+        <v>152491.43835616438</v>
       </c>
       <c r="I23" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="J23">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="K23" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4379,19 +4397,19 @@
       </c>
       <c r="G24" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H24" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>203305.4794520548</v>
+        <v>203549.04109589042</v>
       </c>
       <c r="I24" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="J24">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="K24" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4419,19 +4437,19 @@
       </c>
       <c r="G25" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H25" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>203305.4794520548</v>
+        <v>203549.04109589042</v>
       </c>
       <c r="I25" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="J25">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="K25" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4459,19 +4477,19 @@
       </c>
       <c r="G26" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H26" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>102972.60273972603</v>
+        <v>103106.8493150685</v>
       </c>
       <c r="I26" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="J26">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="K26" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4499,19 +4517,19 @@
       </c>
       <c r="G27" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H27" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>102589.04109589041</v>
+        <v>102723.28767123287</v>
       </c>
       <c r="I27" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="J27">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="K27" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4539,19 +4557,19 @@
       </c>
       <c r="G28" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H28" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>204487.67123287672</v>
+        <v>204756.16438356164</v>
       </c>
       <c r="I28" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>429</v>
+        <v>422</v>
       </c>
       <c r="J28">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="K28" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4579,19 +4597,19 @@
       </c>
       <c r="G29" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H29" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>204065.75342465754</v>
+        <v>204334.24657534246</v>
       </c>
       <c r="I29" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>440</v>
+        <v>433</v>
       </c>
       <c r="J29">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="K29" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4619,19 +4637,19 @@
       </c>
       <c r="G30" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H30" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>102013.69863013699</v>
+        <v>102147.94520547945</v>
       </c>
       <c r="I30" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="J30">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="K30" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4659,19 +4677,19 @@
       </c>
       <c r="G31" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H31" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>101860.27397260274</v>
+        <v>101994.52054794521</v>
       </c>
       <c r="I31" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="J31">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="K31" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4699,19 +4717,19 @@
       </c>
       <c r="G32" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H32" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>204027.39726027398</v>
+        <v>204295.89041095891</v>
       </c>
       <c r="I32" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="J32">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="K32" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4739,19 +4757,19 @@
       </c>
       <c r="G33" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H33" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>101726.02739726027</v>
+        <v>101860.27397260274</v>
       </c>
       <c r="I33" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="J33">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="K33" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4779,19 +4797,19 @@
       </c>
       <c r="G34" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H34" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>215868.76712328766</v>
+        <v>216116.16438356164</v>
       </c>
       <c r="I34" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>462</v>
+        <v>455</v>
       </c>
       <c r="J34">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="K34" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4819,19 +4837,19 @@
       </c>
       <c r="G35" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H35" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>152147.05479452055</v>
+        <v>152332.60273972602</v>
       </c>
       <c r="I35" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="J35">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="K35" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4859,19 +4877,19 @@
       </c>
       <c r="G36" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="H36" s="1">
         <f ca="1">(Table4[[#This Row],[invested days]]/36500*Table4[[#This Row],[Interest Rate]]*Table4[[#This Row],[Invested]]) + Table4[[#This Row],[Invested]]</f>
-        <v>214879.17808219179</v>
+        <v>215126.57534246575</v>
       </c>
       <c r="I36" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>493</v>
+        <v>486</v>
       </c>
       <c r="J36">
         <f ca="1">_xlfn.NUMBERVALUE(Table4[[#This Row],[TODAY]]-Table4[[#This Row],[Created Date]])</f>
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="K36" s="1">
         <f t="shared" ca="1" si="2"/>
@@ -4886,7 +4904,7 @@
       </c>
       <c r="H39" s="5">
         <f ca="1">SUM(Table4[Current Amount])</f>
-        <v>4707387.3958356157</v>
+        <v>4713240.9151232885</v>
       </c>
     </row>
   </sheetData>
@@ -4900,7 +4918,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="9.21875" customWidth="1"/>
@@ -4911,7 +4929,7 @@
     <col min="9" max="9" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -4942,8 +4960,11 @@
       <c r="J1" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="28.8">
+      <c r="K1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="28.8">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -4957,11 +4978,10 @@
         <v>116</v>
       </c>
       <c r="E2" s="2">
-        <f>330000/Table5[[#This Row],[Quantity]]</f>
-        <v>24376.73130193906</v>
+        <v>24376.731301938999</v>
       </c>
       <c r="F2" s="2">
-        <v>29647.1528575958</v>
+        <v>29789.538942108102</v>
       </c>
       <c r="G2" s="2">
         <v>13.5375</v>
@@ -4971,14 +4991,18 @@
       </c>
       <c r="I2" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>330000</v>
+        <v>329999.99999999919</v>
       </c>
       <c r="J2" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>401348.33180970314</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="28.8">
+        <v>403275.88342878839</v>
+      </c>
+      <c r="K2">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>5412.8076401691033</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="28.8">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -4986,7 +5010,7 @@
         <v>118</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>120</v>
@@ -4995,7 +5019,7 @@
         <v>999.33333300000004</v>
       </c>
       <c r="F3" s="2">
-        <v>1998.6</v>
+        <v>1924.3</v>
       </c>
       <c r="G3" s="2">
         <v>9</v>
@@ -5009,231 +5033,259 @@
       </c>
       <c r="J3" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>17987.399999999998</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="28.8">
+        <v>17318.7</v>
+      </c>
+      <c r="K3">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>924.96666699999992</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="28.8">
       <c r="A4" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>125</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E4" s="2">
-        <v>821.43</v>
+        <v>1200.7874999999999</v>
       </c>
       <c r="F4" s="2">
-        <v>1068.45</v>
+        <v>1764.4</v>
       </c>
       <c r="G4" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I4" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>10678.59</v>
+        <v>14409.449999999999</v>
       </c>
       <c r="J4" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>13889.85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="28.8">
+        <v>21172.800000000003</v>
+      </c>
+      <c r="K4">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>563.61250000000018</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="28.8">
       <c r="A5" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E5" s="2">
-        <v>358.558108108108</v>
+        <v>821.43</v>
       </c>
       <c r="F5" s="2">
-        <v>431.35</v>
+        <v>1096</v>
       </c>
       <c r="G5" s="2">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I5" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>11832.417567567563</v>
+        <v>12321.449999999999</v>
       </c>
       <c r="J5" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>14234.550000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="28.8">
+        <v>16440</v>
+      </c>
+      <c r="K5">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>274.57000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="28.8">
       <c r="A6" s="2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>119</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E6" s="2">
-        <v>1200.7874999999999</v>
+        <v>647.45714199999998</v>
       </c>
       <c r="F6" s="2">
-        <v>1764.55</v>
+        <v>829.95</v>
       </c>
       <c r="G6" s="2">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I6" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>14409.449999999999</v>
+        <v>13596.599982</v>
       </c>
       <c r="J6" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>21174.6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="28.8">
+        <v>17428.95</v>
+      </c>
+      <c r="K6">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>182.49285800000007</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="28.8">
       <c r="A7" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>125</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E7" s="2">
-        <v>465.75909090908999</v>
+        <v>234.55245600000001</v>
       </c>
       <c r="F7" s="2">
-        <v>572.75</v>
+        <v>385.95</v>
       </c>
       <c r="G7" s="2">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I7" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>9780.9409090908903</v>
+        <v>13369.489992000001</v>
       </c>
       <c r="J7" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>12027.75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="28.8">
+        <v>21999.149999999998</v>
+      </c>
+      <c r="K7">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>151.39754399999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="28.8">
       <c r="A8" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E8" s="2">
-        <v>234.55245600000001</v>
+        <v>967.73666600000001</v>
       </c>
       <c r="F8" s="2">
-        <v>352.41</v>
+        <v>1110.25</v>
       </c>
       <c r="G8" s="2">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I8" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>13369.489992000001</v>
+        <v>14516.04999</v>
       </c>
       <c r="J8" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>20087.370000000003</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="28.8">
+        <v>16653.75</v>
+      </c>
+      <c r="K8">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>142.51333399999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="28.8">
       <c r="A9" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E9" s="2">
-        <v>647.45714199999998</v>
+        <v>465.75909000000001</v>
       </c>
       <c r="F9" s="2">
-        <v>813.35</v>
+        <v>587.6</v>
       </c>
       <c r="G9" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I9" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>13596.599982</v>
+        <v>10246.699980000001</v>
       </c>
       <c r="J9" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>17080.350000000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="28.8">
+        <v>12927.2</v>
+      </c>
+      <c r="K9">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>121.84091000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="28.8">
       <c r="A10" s="2">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="E10" s="2">
-        <v>967.736666666666</v>
+        <v>1066.3</v>
       </c>
       <c r="F10" s="2">
-        <v>1096.3499999999999</v>
+        <v>1177.5999999999999</v>
       </c>
       <c r="G10" s="2">
         <v>14</v>
@@ -5243,184 +5295,208 @@
       </c>
       <c r="I10" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>13548.313333333324</v>
+        <v>14928.199999999999</v>
       </c>
       <c r="J10" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>15348.899999999998</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="28.8">
+        <v>16486.399999999998</v>
+      </c>
+      <c r="K10">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>111.29999999999995</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="28.8">
       <c r="A11" s="2">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="E11" s="2">
-        <v>287.445098039215</v>
+        <v>1356.986666</v>
       </c>
       <c r="F11" s="2">
-        <v>318.35000000000002</v>
+        <v>1450</v>
       </c>
       <c r="G11" s="2">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I11" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>14372.25490196075</v>
+        <v>20354.79999</v>
       </c>
       <c r="J11" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>15917.500000000002</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="28.8">
+        <v>21750</v>
+      </c>
+      <c r="K11">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>93.013333999999986</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="28.8">
       <c r="A12" s="2">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>119</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E12" s="2">
-        <v>439.73939300000001</v>
+        <v>358.558108</v>
       </c>
       <c r="F12" s="2">
-        <v>488.9</v>
+        <v>438.15</v>
       </c>
       <c r="G12" s="2">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I12" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>14511.399969</v>
+        <v>13266.649996</v>
       </c>
       <c r="J12" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>16133.699999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="28.8">
+        <v>16211.55</v>
+      </c>
+      <c r="K12">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>79.591891999999973</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="28.8">
       <c r="A13" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E13" s="2">
-        <v>42.077151515151499</v>
+        <v>439.73939300000001</v>
       </c>
       <c r="F13" s="2">
-        <v>41.75</v>
+        <v>500.1</v>
       </c>
       <c r="G13" s="2">
-        <v>311</v>
+        <v>33</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I13" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>13085.994121212116</v>
+        <v>14511.399969</v>
       </c>
       <c r="J13" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>12984.25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="28.8">
+        <v>16503.3</v>
+      </c>
+      <c r="K13">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>60.360607000000016</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="28.8">
       <c r="A14" s="2">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>119</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E14" s="2">
-        <v>156.610434</v>
+        <v>172.61421000000001</v>
       </c>
       <c r="F14" s="2">
-        <v>184.7</v>
+        <v>210.75</v>
       </c>
       <c r="G14" s="2">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I14" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>14408.159927999999</v>
+        <v>16398.34995</v>
       </c>
       <c r="J14" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>16992.399999999998</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="28.8">
+        <v>20021.25</v>
+      </c>
+      <c r="K14">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>38.135789999999986</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="28.8">
       <c r="A15" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>125</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E15" s="2">
-        <v>1066.3</v>
+        <v>156.610434</v>
       </c>
       <c r="F15" s="2">
-        <v>1100.95</v>
+        <v>186.04</v>
       </c>
       <c r="G15" s="2">
-        <v>14</v>
+        <v>92</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I15" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>14928.199999999999</v>
+        <v>14408.159927999999</v>
       </c>
       <c r="J15" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>15413.300000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="28.8">
+        <v>17115.68</v>
+      </c>
+      <c r="K15">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>29.429565999999994</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="28.8">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -5434,61 +5510,69 @@
         <v>148</v>
       </c>
       <c r="E16" s="2">
-        <v>785.48333333333301</v>
+        <v>785.48333300000002</v>
       </c>
       <c r="F16" s="2">
-        <v>775</v>
+        <v>814.8</v>
       </c>
       <c r="G16" s="2">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I16" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>14924.183333333327</v>
+        <v>16495.149992999999</v>
       </c>
       <c r="J16" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>14725</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="28.8">
+        <v>17110.8</v>
+      </c>
+      <c r="K16">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>29.316666999999939</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="28.8">
       <c r="A17" s="2">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E17" s="2">
-        <v>172.61421000000001</v>
+        <v>287.44509799999997</v>
       </c>
       <c r="F17" s="2">
-        <v>215.1</v>
+        <v>315.95</v>
       </c>
       <c r="G17" s="2">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I17" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>16398.34995</v>
+        <v>14659.699997999998</v>
       </c>
       <c r="J17" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>20434.5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="28.8">
+        <v>16113.449999999999</v>
+      </c>
+      <c r="K17">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>28.504902000000016</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="28.8">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -5496,135 +5580,151 @@
         <v>151</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>152</v>
       </c>
       <c r="E18" s="2">
-        <v>253.726078431372</v>
+        <v>253.726078</v>
       </c>
       <c r="F18" s="2">
-        <v>253.24</v>
+        <v>256.39999999999998</v>
       </c>
       <c r="G18" s="2">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I18" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>12432.577843137227</v>
+        <v>12940.029978</v>
       </c>
       <c r="J18" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>12408.76</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="28.8">
+        <v>13076.4</v>
+      </c>
+      <c r="K18">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>2.6739219999999762</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="28.8">
       <c r="A19" s="2">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="E19" s="2">
-        <v>172.755490196078</v>
+        <v>42.077151000000001</v>
       </c>
       <c r="F19" s="2">
-        <v>162.1</v>
+        <v>41.85</v>
       </c>
       <c r="G19" s="2">
-        <v>97</v>
+        <v>330</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I19" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>16757.282549019565</v>
+        <v>13885.45983</v>
       </c>
       <c r="J19" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>15723.699999999999</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="28.8">
+        <v>13810.5</v>
+      </c>
+      <c r="K19">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>-0.22715099999999921</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="28.8">
       <c r="A20" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E20" s="2">
-        <v>1356.986666</v>
+        <v>69.901465999999999</v>
       </c>
       <c r="F20" s="2">
-        <v>1414.4</v>
+        <v>69.58</v>
       </c>
       <c r="G20" s="2">
-        <v>15</v>
+        <v>341</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I20" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>20354.79999</v>
+        <v>23836.399905999999</v>
       </c>
       <c r="J20" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>21216</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="28.8">
+        <v>23726.78</v>
+      </c>
+      <c r="K20">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>-0.32146600000000092</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="28.8">
       <c r="A21" s="2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>119</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E21" s="2">
-        <v>69.9014662756598</v>
+        <v>172.75549000000001</v>
       </c>
       <c r="F21" s="2">
-        <v>69.64</v>
+        <v>167.9</v>
       </c>
       <c r="G21" s="2">
-        <v>337</v>
+        <v>102</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I21" s="1">
         <f>Table5[[#This Row],[Average Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>23556.794134897351</v>
+        <v>17621.059980000002</v>
       </c>
       <c r="J21" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>23468.68</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="28.8">
+        <v>17125.8</v>
+      </c>
+      <c r="K21">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>-4.8554900000000032</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="28.8">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -5641,7 +5741,7 @@
         <v>1217.328571</v>
       </c>
       <c r="F22" s="2">
-        <v>1117.6500000000001</v>
+        <v>1185</v>
       </c>
       <c r="G22" s="2">
         <v>14</v>
@@ -5655,17 +5755,29 @@
       </c>
       <c r="J22" s="1">
         <f>Table5[[#This Row],[Current Price]]*Table5[[#This Row],[Quantity]]</f>
-        <v>15647.100000000002</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10">
+        <v>16590</v>
+      </c>
+      <c r="K22">
+        <f>Table5[[#This Row],[Current Price]]-Table5[[#This Row],[Average Price]]</f>
+        <v>-32.328571000000011</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="H25">
+        <f>I25-I2</f>
+        <v>297801.69945299998</v>
+      </c>
       <c r="I25">
         <f>SUM(Table5[Invested])</f>
-        <v>618982.39849555213</v>
+        <v>627801.69945299916</v>
       </c>
       <c r="J25">
         <f>SUM(Table5[current])</f>
-        <v>734243.99180970306</v>
+        <v>752858.34342878871</v>
+      </c>
+      <c r="K25">
+        <f>J25-J2</f>
+        <v>349582.46000000031</v>
       </c>
     </row>
   </sheetData>
@@ -5679,11 +5791,12 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="3" max="3" width="12.6640625" customWidth="1"/>
     <col min="4" max="4" width="14.44140625" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" customWidth="1"/>
     <col min="7" max="7" width="15.5546875" customWidth="1"/>
     <col min="8" max="8" width="11.5546875" customWidth="1"/>
@@ -5691,7 +5804,7 @@
     <col min="11" max="12" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -5729,7 +5842,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="57.6">
+    <row r="2" spans="1:13" ht="57.6">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -5749,10 +5862,10 @@
         <v>40.19</v>
       </c>
       <c r="G2" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H2" s="2">
-        <v>40.978099999999998</v>
+        <v>41.029000000000003</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2">
@@ -5764,10 +5877,10 @@
       </c>
       <c r="L2" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>21409.254213600001</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="57.6">
+        <v>21435.847224000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="57.6">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -5781,16 +5894,16 @@
         <v>120828</v>
       </c>
       <c r="E3" s="2">
-        <v>369.96</v>
+        <v>380.53699999999998</v>
       </c>
       <c r="F3" s="2">
-        <v>256.77</v>
+        <v>257.52</v>
       </c>
       <c r="G3" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H3" s="2">
-        <v>280.4819</v>
+        <v>292.1925</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2">
@@ -5798,14 +5911,14 @@
       </c>
       <c r="K3" s="2">
         <f>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</f>
-        <v>94994.629199999981</v>
+        <v>97995.888239999986</v>
       </c>
       <c r="L3" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>103767.083724</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="57.6">
+        <v>111190.05737249998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="57.6">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -5819,16 +5932,16 @@
         <v>118778</v>
       </c>
       <c r="E4" s="2">
-        <v>505.26499999999999</v>
+        <v>520.36699999999996</v>
       </c>
       <c r="F4" s="2">
-        <v>174.16</v>
+        <v>174.87</v>
       </c>
       <c r="G4" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H4" s="2">
-        <v>192.0823</v>
+        <v>198.3537</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2">
@@ -5836,14 +5949,14 @@
       </c>
       <c r="K4" s="2">
         <f>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</f>
-        <v>87996.952399999995</v>
+        <v>90996.577290000001</v>
       </c>
       <c r="L4" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>97052.463309500003</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="72">
+        <v>103216.71980789999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="72">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -5857,16 +5970,16 @@
         <v>118968</v>
       </c>
       <c r="E5" s="2">
-        <v>186.92</v>
+        <v>192.21799999999999</v>
       </c>
       <c r="F5" s="2">
-        <v>513.55999999999995</v>
+        <v>515.01</v>
       </c>
       <c r="G5" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H5" s="2">
-        <v>558.92200000000003</v>
+        <v>562.96799999999996</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2">
@@ -5874,14 +5987,14 @@
       </c>
       <c r="K5" s="2">
         <f>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</f>
-        <v>95994.63519999999</v>
+        <v>98994.192179999998</v>
       </c>
       <c r="L5" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>104473.70023999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="57.6">
+        <v>108212.58302399999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="57.6">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -5895,16 +6008,16 @@
         <v>118979</v>
       </c>
       <c r="E6" s="2">
-        <v>1827.932</v>
+        <v>1884.3679999999999</v>
       </c>
       <c r="F6" s="2">
-        <v>49.26</v>
+        <v>49.38</v>
       </c>
       <c r="G6" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H6" s="2">
-        <v>52.677</v>
+        <v>53.267000000000003</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2">
@@ -5912,14 +6025,14 @@
       </c>
       <c r="K6" s="2">
         <f>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</f>
-        <v>90043.930319999999</v>
+        <v>93050.091840000008</v>
       </c>
       <c r="L6" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>96289.973964000004</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="43.2">
+        <v>100374.630256</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="43.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -5933,16 +6046,16 @@
         <v>125307</v>
       </c>
       <c r="E7" s="2">
-        <v>1115.356</v>
+        <v>1155.152</v>
       </c>
       <c r="F7" s="2">
-        <v>67.239999999999995</v>
+        <v>67.52</v>
       </c>
       <c r="G7" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H7" s="2">
-        <v>72.930000000000007</v>
+        <v>75.209999999999994</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2">
@@ -5950,14 +6063,14 @@
       </c>
       <c r="K7" s="2">
         <f>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</f>
-        <v>74996.53744</v>
+        <v>77995.863039999997</v>
       </c>
       <c r="L7" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>81342.913080000013</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="72">
+        <v>86878.981919999991</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="72">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -5971,16 +6084,16 @@
         <v>149219</v>
       </c>
       <c r="E8" s="2">
-        <v>3624.2379999999998</v>
+        <v>3755.5439999999999</v>
       </c>
       <c r="F8" s="2">
-        <v>15.45</v>
+        <v>15.71</v>
       </c>
       <c r="G8" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H8" s="2">
-        <v>22.752600000000001</v>
+        <v>24.0243</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2">
@@ -5988,14 +6101,14 @@
       </c>
       <c r="K8" s="2">
         <f>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</f>
-        <v>55994.477099999996</v>
+        <v>58999.596239999999</v>
       </c>
       <c r="L8" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>82460.837518800006</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="57.6">
+        <v>90224.315719199993</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="57.6">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -6009,16 +6122,16 @@
         <v>118482</v>
       </c>
       <c r="E9" s="2">
-        <v>1447.414</v>
+        <v>1503.3320000000001</v>
       </c>
       <c r="F9" s="2">
-        <v>51.12</v>
+        <v>51.22</v>
       </c>
       <c r="G9" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H9" s="2">
-        <v>53.3767</v>
+        <v>53.772599999999997</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2">
@@ -6026,14 +6139,14 @@
       </c>
       <c r="K9" s="2">
         <f>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</f>
-        <v>73991.803679999997</v>
+        <v>77000.665040000007</v>
       </c>
       <c r="L9" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>77258.182853799997</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="72">
+        <v>80838.070303200002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="72">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -6047,16 +6160,16 @@
         <v>147662</v>
       </c>
       <c r="E10" s="2">
-        <v>1792.5029999999999</v>
+        <v>1849.308</v>
       </c>
       <c r="F10" s="2">
-        <v>41.84</v>
+        <v>42.18</v>
       </c>
       <c r="G10" s="18">
-        <v>46144.142696759256</v>
+        <v>46149.092395833337</v>
       </c>
       <c r="H10" s="2">
-        <v>51.32</v>
+        <v>52.39</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2">
@@ -6064,14 +6177,14 @@
       </c>
       <c r="K10" s="2">
         <f>Table7[[#This Row],[average_nav]]*Table7[[#This Row],[units]]</f>
-        <v>74998.325519999999</v>
+        <v>78003.811440000005</v>
       </c>
       <c r="L10" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>91991.253960000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+        <v>96885.246119999996</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -6090,7 +6203,7 @@
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2">
-        <v>205126.91</v>
+        <v>206981.26</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2">
@@ -6102,17 +6215,25 @@
       </c>
       <c r="L11" s="2">
         <f>Table7[[#This Row],[latest_nav]]*Table7[[#This Row],[units]]</f>
-        <v>205126.91</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
+        <v>206981.26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="J13">
+        <f>K13-K11</f>
+        <v>694034.19194999989</v>
+      </c>
       <c r="K13">
         <f>SUM(Table7[Invested])</f>
-        <v>873313.89749999985</v>
+        <v>897339.29194999987</v>
       </c>
       <c r="L13">
         <f>SUM(Table7[Current])</f>
-        <v>961172.5728637001</v>
+        <v>1006237.7117467999</v>
+      </c>
+      <c r="M13">
+        <f>L13-L11</f>
+        <v>799256.45174679987</v>
       </c>
     </row>
   </sheetData>
@@ -6262,7 +6383,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="10.6640625" customWidth="1"/>
@@ -6348,7 +6469,7 @@
         <v>167</v>
       </c>
       <c r="C6" s="3">
-        <v>-350388.25</v>
+        <v>-322647.55</v>
       </c>
       <c r="D6" s="1">
         <v>8.35</v>
@@ -6387,9 +6508,12 @@
       <c r="A9" s="1"/>
       <c r="C9" s="1">
         <f>SUM(Table9[Amount])</f>
-        <v>3336602.75</v>
+        <v>3364343.45</v>
       </c>
       <c r="D9" s="1"/>
+    </row>
+    <row r="20" spans="3:3">
+      <c r="C20" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>